<commit_message>
add: Nueva Data y modulos.
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/clientes.xlsx
+++ b/api/src/main/resources/importaciones/clientes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6460AF6-901A-44C3-92D3-3DF959EC20DC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9CD8B5E-D1D8-42DE-8EC3-C666A375E1D3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="120" yWindow="120" windowWidth="18915" windowHeight="8475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="128">
   <si>
     <t>cliente</t>
   </si>
@@ -373,9 +373,6 @@
     <t>tipoCliente</t>
   </si>
   <si>
-    <t>PN</t>
-  </si>
-  <si>
     <t>S</t>
   </si>
   <si>
@@ -386,13 +383,34 @@
   </si>
   <si>
     <t>Es Proveedor</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>Provincia</t>
+  </si>
+  <si>
+    <t>Canton</t>
+  </si>
+  <si>
+    <t>Parroquia</t>
+  </si>
+  <si>
+    <t>Sexo</t>
+  </si>
+  <si>
+    <t>Estado Civil</t>
+  </si>
+  <si>
+    <t>Origen de Ingresos</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -430,6 +448,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -440,17 +464,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="13"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -461,14 +500,17 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -876,61 +918,81 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:S23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="106.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="33.7109375" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="59.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="31.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.85546875" customWidth="1"/>
-    <col min="12" max="13" width="17.7109375" customWidth="1"/>
+    <col min="5" max="5" width="59.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="17" width="21.85546875" customWidth="1"/>
+    <col min="18" max="19" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="K1" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="S1" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -940,38 +1002,46 @@
       <c r="C2" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
-        <v>117</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L2" t="s">
-        <v>118</v>
-      </c>
-      <c r="M2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>121</v>
+      </c>
+      <c r="L2" s="5">
+        <v>10</v>
+      </c>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" t="s">
+        <v>117</v>
+      </c>
+      <c r="S2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -981,26 +1051,29 @@
       <c r="C3" t="s">
         <v>40</v>
       </c>
+      <c r="E3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" t="s">
+        <v>77</v>
+      </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="H3" t="s">
-        <v>77</v>
-      </c>
-      <c r="I3" t="s">
-        <v>84</v>
-      </c>
-      <c r="J3" t="s">
         <v>101</v>
       </c>
-      <c r="L3" t="s">
-        <v>118</v>
-      </c>
-      <c r="M3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K3" t="s">
+        <v>118</v>
+      </c>
+      <c r="R3" t="s">
+        <v>117</v>
+      </c>
+      <c r="S3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1010,26 +1083,29 @@
       <c r="C4" t="s">
         <v>41</v>
       </c>
+      <c r="E4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
       <c r="G4" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="H4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" t="s">
-        <v>83</v>
-      </c>
-      <c r="J4" t="s">
         <v>100</v>
       </c>
-      <c r="L4" t="s">
-        <v>119</v>
-      </c>
-      <c r="M4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K4" t="s">
+        <v>121</v>
+      </c>
+      <c r="R4" t="s">
+        <v>118</v>
+      </c>
+      <c r="S4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -1039,26 +1115,29 @@
       <c r="C5" t="s">
         <v>42</v>
       </c>
+      <c r="E5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" t="s">
+        <v>77</v>
+      </c>
       <c r="G5" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="H5" t="s">
-        <v>77</v>
-      </c>
-      <c r="I5" t="s">
-        <v>85</v>
-      </c>
-      <c r="J5" t="s">
         <v>102</v>
       </c>
-      <c r="L5" t="s">
-        <v>118</v>
-      </c>
-      <c r="M5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K5" t="s">
+        <v>118</v>
+      </c>
+      <c r="R5" t="s">
+        <v>117</v>
+      </c>
+      <c r="S5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1068,26 +1147,26 @@
       <c r="C6" t="s">
         <v>43</v>
       </c>
+      <c r="E6" t="s">
+        <v>114</v>
+      </c>
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
       <c r="G6" t="s">
-        <v>114</v>
+        <v>86</v>
       </c>
       <c r="H6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I6" t="s">
-        <v>86</v>
-      </c>
-      <c r="J6" t="s">
         <v>103</v>
       </c>
-      <c r="L6" t="s">
-        <v>118</v>
-      </c>
-      <c r="M6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R6" t="s">
+        <v>117</v>
+      </c>
+      <c r="S6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1097,26 +1176,26 @@
       <c r="C7" t="s">
         <v>44</v>
       </c>
+      <c r="E7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7" t="s">
+        <v>78</v>
+      </c>
       <c r="G7" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="H7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I7" t="s">
-        <v>87</v>
-      </c>
-      <c r="J7" t="s">
         <v>104</v>
       </c>
-      <c r="L7" t="s">
-        <v>119</v>
-      </c>
-      <c r="M7" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R7" t="s">
+        <v>118</v>
+      </c>
+      <c r="S7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1126,26 +1205,26 @@
       <c r="C8" t="s">
         <v>45</v>
       </c>
+      <c r="E8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" t="s">
+        <v>79</v>
+      </c>
       <c r="G8" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="H8" t="s">
-        <v>79</v>
-      </c>
-      <c r="I8" t="s">
-        <v>88</v>
-      </c>
-      <c r="J8" t="s">
         <v>105</v>
       </c>
-      <c r="L8" t="s">
-        <v>118</v>
-      </c>
-      <c r="M8" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R8" t="s">
+        <v>117</v>
+      </c>
+      <c r="S8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -1155,26 +1234,26 @@
       <c r="C9" t="s">
         <v>46</v>
       </c>
+      <c r="E9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" t="s">
+        <v>80</v>
+      </c>
       <c r="G9" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="H9" t="s">
-        <v>80</v>
-      </c>
-      <c r="I9" t="s">
-        <v>89</v>
-      </c>
-      <c r="J9" t="s">
         <v>106</v>
       </c>
-      <c r="L9" t="s">
-        <v>119</v>
-      </c>
-      <c r="M9" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R9" t="s">
+        <v>118</v>
+      </c>
+      <c r="S9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1184,27 +1263,27 @@
       <c r="C10" t="s">
         <v>47</v>
       </c>
+      <c r="E10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" t="s">
+        <v>81</v>
+      </c>
       <c r="G10" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="H10" t="s">
-        <v>81</v>
-      </c>
-      <c r="I10" t="s">
-        <v>90</v>
-      </c>
-      <c r="J10" t="s">
         <v>107</v>
       </c>
-      <c r="L10" t="s">
-        <v>118</v>
-      </c>
-      <c r="M10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="R10" t="s">
+        <v>117</v>
+      </c>
+      <c r="S10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -1213,55 +1292,55 @@
       <c r="C11" t="s">
         <v>48</v>
       </c>
+      <c r="E11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="G11" t="s">
-        <v>66</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" t="s">
         <v>91</v>
       </c>
-      <c r="J11" t="s">
+      <c r="H11" t="s">
         <v>108</v>
       </c>
-      <c r="L11" t="s">
-        <v>119</v>
-      </c>
-      <c r="M11" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R11" t="s">
+        <v>118</v>
+      </c>
+      <c r="S11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>30</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>49</v>
       </c>
+      <c r="E12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" t="s">
+        <v>20</v>
+      </c>
       <c r="G12" t="s">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="H12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" t="s">
-        <v>92</v>
-      </c>
-      <c r="J12" t="s">
         <v>76</v>
       </c>
-      <c r="L12" t="s">
-        <v>118</v>
-      </c>
-      <c r="M12" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R12" t="s">
+        <v>117</v>
+      </c>
+      <c r="S12" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1271,26 +1350,26 @@
       <c r="C13" t="s">
         <v>50</v>
       </c>
+      <c r="E13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" t="s">
+        <v>20</v>
+      </c>
       <c r="G13" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="H13" t="s">
-        <v>20</v>
-      </c>
-      <c r="I13" t="s">
-        <v>93</v>
-      </c>
-      <c r="J13" t="s">
         <v>76</v>
       </c>
-      <c r="L13" t="s">
-        <v>118</v>
-      </c>
-      <c r="M13" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R13" t="s">
+        <v>117</v>
+      </c>
+      <c r="S13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1300,27 +1379,27 @@
       <c r="C14" t="s">
         <v>51</v>
       </c>
+      <c r="E14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
+      </c>
       <c r="G14" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="H14" t="s">
-        <v>20</v>
-      </c>
-      <c r="I14" t="s">
-        <v>94</v>
-      </c>
-      <c r="J14" t="s">
         <v>109</v>
       </c>
-      <c r="L14" t="s">
-        <v>118</v>
-      </c>
-      <c r="M14" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="R14" t="s">
+        <v>117</v>
+      </c>
+      <c r="S14" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -1329,26 +1408,26 @@
       <c r="C15" t="s">
         <v>52</v>
       </c>
+      <c r="E15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" t="s">
+        <v>20</v>
+      </c>
       <c r="G15" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="H15" t="s">
-        <v>20</v>
-      </c>
-      <c r="I15" t="s">
-        <v>76</v>
-      </c>
-      <c r="J15" t="s">
         <v>110</v>
       </c>
-      <c r="L15" t="s">
-        <v>119</v>
-      </c>
-      <c r="M15" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R15" t="s">
+        <v>118</v>
+      </c>
+      <c r="S15" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -1358,26 +1437,26 @@
       <c r="C16" t="s">
         <v>53</v>
       </c>
+      <c r="E16" t="s">
+        <v>114</v>
+      </c>
+      <c r="F16" t="s">
+        <v>82</v>
+      </c>
       <c r="G16" t="s">
-        <v>114</v>
+        <v>76</v>
       </c>
       <c r="H16" t="s">
-        <v>82</v>
-      </c>
-      <c r="I16" t="s">
         <v>76</v>
       </c>
-      <c r="J16" t="s">
-        <v>76</v>
-      </c>
-      <c r="L16" t="s">
-        <v>118</v>
-      </c>
-      <c r="M16" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R16" t="s">
+        <v>117</v>
+      </c>
+      <c r="S16" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -1387,26 +1466,26 @@
       <c r="C17" t="s">
         <v>54</v>
       </c>
+      <c r="E17" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" t="s">
+        <v>20</v>
+      </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="H17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I17" t="s">
-        <v>95</v>
-      </c>
-      <c r="J17" t="s">
         <v>76</v>
       </c>
-      <c r="L17" t="s">
-        <v>118</v>
-      </c>
-      <c r="M17" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R17" t="s">
+        <v>117</v>
+      </c>
+      <c r="S17" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -1416,26 +1495,26 @@
       <c r="C18" t="s">
         <v>55</v>
       </c>
+      <c r="E18" t="s">
+        <v>72</v>
+      </c>
+      <c r="F18" t="s">
+        <v>20</v>
+      </c>
       <c r="G18" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="H18" t="s">
-        <v>20</v>
-      </c>
-      <c r="I18" t="s">
-        <v>96</v>
-      </c>
-      <c r="J18" t="s">
         <v>76</v>
       </c>
-      <c r="L18" t="s">
-        <v>118</v>
-      </c>
-      <c r="M18" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R18" t="s">
+        <v>117</v>
+      </c>
+      <c r="S18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1445,26 +1524,26 @@
       <c r="C19" t="s">
         <v>56</v>
       </c>
+      <c r="E19" t="s">
+        <v>73</v>
+      </c>
+      <c r="F19" t="s">
+        <v>20</v>
+      </c>
       <c r="G19" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="H19" t="s">
-        <v>20</v>
-      </c>
-      <c r="I19" t="s">
-        <v>97</v>
-      </c>
-      <c r="J19" t="s">
         <v>111</v>
       </c>
-      <c r="L19" t="s">
-        <v>118</v>
-      </c>
-      <c r="M19" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R19" t="s">
+        <v>117</v>
+      </c>
+      <c r="S19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -1474,26 +1553,26 @@
       <c r="C20" t="s">
         <v>57</v>
       </c>
+      <c r="E20" t="s">
+        <v>74</v>
+      </c>
+      <c r="F20" t="s">
+        <v>20</v>
+      </c>
       <c r="G20" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="H20" t="s">
-        <v>20</v>
-      </c>
-      <c r="I20" t="s">
-        <v>98</v>
-      </c>
-      <c r="J20" t="s">
         <v>112</v>
       </c>
-      <c r="L20" t="s">
-        <v>118</v>
-      </c>
-      <c r="M20" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="R20" t="s">
+        <v>117</v>
+      </c>
+      <c r="S20" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -1503,23 +1582,82 @@
       <c r="C21" t="s">
         <v>58</v>
       </c>
+      <c r="E21" t="s">
+        <v>75</v>
+      </c>
+      <c r="F21" t="s">
+        <v>20</v>
+      </c>
       <c r="G21" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="H21" t="s">
-        <v>20</v>
-      </c>
-      <c r="I21" t="s">
-        <v>99</v>
-      </c>
-      <c r="J21" t="s">
         <v>113</v>
       </c>
-      <c r="L21" t="s">
-        <v>118</v>
-      </c>
-      <c r="M21" t="s">
-        <v>119</v>
+      <c r="R21" t="s">
+        <v>117</v>
+      </c>
+      <c r="S21" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>0</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23">
+        <v>4</v>
+      </c>
+      <c r="F23">
+        <v>5</v>
+      </c>
+      <c r="G23">
+        <v>6</v>
+      </c>
+      <c r="H23">
+        <v>7</v>
+      </c>
+      <c r="I23">
+        <v>8</v>
+      </c>
+      <c r="J23">
+        <v>9</v>
+      </c>
+      <c r="K23">
+        <v>10</v>
+      </c>
+      <c r="L23">
+        <v>11</v>
+      </c>
+      <c r="M23">
+        <v>12</v>
+      </c>
+      <c r="N23">
+        <v>13</v>
+      </c>
+      <c r="O23">
+        <v>14</v>
+      </c>
+      <c r="P23">
+        <v>15</v>
+      </c>
+      <c r="Q23">
+        <v>16</v>
+      </c>
+      <c r="R23">
+        <v>17</v>
+      </c>
+      <c r="S23">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add: Se quito del request cuentas por cobrar de venta impuestos
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/clientes.xlsx
+++ b/api/src/main/resources/importaciones/clientes.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5169FA8-CA39-49BC-9098-239F1959A885}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8611FB71-A9F3-47C6-A0DA-DE0D701204D8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="120" yWindow="120" windowWidth="18915" windowHeight="8475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" refMode="R1C1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="130">
   <si>
     <t>cliente</t>
   </si>
@@ -407,6 +407,9 @@
   </si>
   <si>
     <t>Pais</t>
+  </si>
+  <si>
+    <t>Codigo Tercero</t>
   </si>
 </sst>
 </file>
@@ -912,23 +915,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T23"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="106.7109375" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.7109375" customWidth="1"/>
-    <col min="5" max="5" width="59.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="31.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.85546875" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" customWidth="1"/>
-    <col min="13" max="18" width="21.85546875" customWidth="1"/>
-    <col min="19" max="20" width="17.7109375" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" customWidth="1"/>
+    <col min="5" max="5" width="33.7109375" customWidth="1"/>
+    <col min="6" max="6" width="59.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.85546875" customWidth="1"/>
+    <col min="11" max="11" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.42578125" customWidth="1"/>
+    <col min="14" max="19" width="21.85546875" customWidth="1"/>
+    <col min="20" max="21" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -939,58 +943,61 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="T1" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="U1" s="6" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1000,46 +1007,47 @@
       <c r="C2" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="1"/>
+      <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>12</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>121</v>
       </c>
-      <c r="M2" s="5">
+      <c r="N2" s="5">
         <v>10</v>
       </c>
-      <c r="N2" s="3"/>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
-      <c r="S2" t="s">
-        <v>117</v>
-      </c>
+      <c r="S2" s="3"/>
       <c r="T2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1049,29 +1057,29 @@
       <c r="C3" t="s">
         <v>40</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>60</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>77</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>84</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>101</v>
       </c>
-      <c r="K3" t="s">
-        <v>118</v>
-      </c>
-      <c r="S3" t="s">
-        <v>117</v>
+      <c r="L3" t="s">
+        <v>118</v>
       </c>
       <c r="T3" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1081,29 +1089,29 @@
       <c r="C4" t="s">
         <v>41</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>61</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>13</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>83</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>100</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>121</v>
       </c>
-      <c r="S4" t="s">
-        <v>118</v>
-      </c>
       <c r="T4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="U4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -1113,29 +1121,29 @@
       <c r="C5" t="s">
         <v>42</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>59</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>77</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>85</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>102</v>
       </c>
-      <c r="K5" t="s">
-        <v>118</v>
-      </c>
-      <c r="S5" t="s">
-        <v>117</v>
+      <c r="L5" t="s">
+        <v>118</v>
       </c>
       <c r="T5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1145,26 +1153,26 @@
       <c r="C6" t="s">
         <v>43</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>114</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>13</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>86</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>103</v>
       </c>
-      <c r="S6" t="s">
-        <v>117</v>
-      </c>
       <c r="T6" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1174,26 +1182,26 @@
       <c r="C7" t="s">
         <v>44</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>62</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>78</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>87</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>104</v>
       </c>
-      <c r="S7" t="s">
-        <v>118</v>
-      </c>
       <c r="T7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="U7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1203,26 +1211,26 @@
       <c r="C8" t="s">
         <v>45</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>63</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>79</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>88</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>105</v>
       </c>
-      <c r="S8" t="s">
-        <v>117</v>
-      </c>
       <c r="T8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -1232,26 +1240,26 @@
       <c r="C9" t="s">
         <v>46</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>64</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>80</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>89</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>106</v>
       </c>
-      <c r="S9" t="s">
-        <v>118</v>
-      </c>
       <c r="T9" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="U9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1261,26 +1269,26 @@
       <c r="C10" t="s">
         <v>47</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>65</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>81</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>90</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>107</v>
       </c>
-      <c r="S10" t="s">
-        <v>117</v>
-      </c>
       <c r="T10" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>29</v>
       </c>
@@ -1290,26 +1298,26 @@
       <c r="C11" t="s">
         <v>48</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>66</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>91</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>108</v>
       </c>
-      <c r="S11" t="s">
-        <v>118</v>
-      </c>
       <c r="T11" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="U11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -1319,26 +1327,27 @@
       <c r="C12" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E12" t="s">
+      <c r="D12" s="4"/>
+      <c r="F12" t="s">
         <v>67</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>20</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>92</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>76</v>
       </c>
-      <c r="S12" t="s">
-        <v>117</v>
-      </c>
       <c r="T12" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U12" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1348,26 +1357,26 @@
       <c r="C13" t="s">
         <v>50</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>68</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>20</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>93</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>76</v>
       </c>
-      <c r="S13" t="s">
-        <v>117</v>
-      </c>
       <c r="T13" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1377,26 +1386,26 @@
       <c r="C14" t="s">
         <v>51</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>69</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>20</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>94</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>109</v>
       </c>
-      <c r="S14" t="s">
-        <v>117</v>
-      </c>
       <c r="T14" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U14" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>33</v>
       </c>
@@ -1406,26 +1415,26 @@
       <c r="C15" t="s">
         <v>52</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>70</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>20</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>76</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>110</v>
       </c>
-      <c r="S15" t="s">
-        <v>118</v>
-      </c>
       <c r="T15" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="U15" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -1435,26 +1444,26 @@
       <c r="C16" t="s">
         <v>53</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>114</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>82</v>
-      </c>
-      <c r="G16" t="s">
-        <v>76</v>
       </c>
       <c r="H16" t="s">
         <v>76</v>
       </c>
-      <c r="S16" t="s">
-        <v>117</v>
+      <c r="I16" t="s">
+        <v>76</v>
       </c>
       <c r="T16" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U16" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -1464,26 +1473,26 @@
       <c r="C17" t="s">
         <v>54</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>71</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>20</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>95</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>76</v>
       </c>
-      <c r="S17" t="s">
-        <v>117</v>
-      </c>
       <c r="T17" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U17" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -1493,26 +1502,26 @@
       <c r="C18" t="s">
         <v>55</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>72</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>20</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>96</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>76</v>
       </c>
-      <c r="S18" t="s">
-        <v>117</v>
-      </c>
       <c r="T18" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1522,26 +1531,26 @@
       <c r="C19" t="s">
         <v>56</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>73</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>20</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>97</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>111</v>
       </c>
-      <c r="S19" t="s">
-        <v>117</v>
-      </c>
       <c r="T19" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="U19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -1551,26 +1560,26 @@
       <c r="C20" t="s">
         <v>57</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>74</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>20</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>98</v>
       </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>112</v>
       </c>
-      <c r="S20" t="s">
-        <v>117</v>
-      </c>
       <c r="T20" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U20" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -1580,90 +1589,28 @@
       <c r="C21" t="s">
         <v>58</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>75</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>20</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>99</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>113</v>
       </c>
-      <c r="S21" t="s">
-        <v>117</v>
-      </c>
       <c r="T21" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>0</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23">
-        <v>2</v>
-      </c>
-      <c r="D23">
-        <v>3</v>
-      </c>
-      <c r="E23">
-        <v>4</v>
-      </c>
-      <c r="F23">
-        <v>5</v>
-      </c>
-      <c r="G23">
-        <v>6</v>
-      </c>
-      <c r="H23">
-        <v>7</v>
-      </c>
-      <c r="I23">
-        <v>8</v>
-      </c>
-      <c r="J23">
-        <v>9</v>
-      </c>
-      <c r="K23">
-        <v>10</v>
-      </c>
-      <c r="L23">
-        <v>11</v>
-      </c>
-      <c r="M23">
-        <v>12</v>
-      </c>
-      <c r="N23">
-        <v>13</v>
-      </c>
-      <c r="O23">
-        <v>14</v>
-      </c>
-      <c r="P23">
-        <v>15</v>
-      </c>
-      <c r="Q23">
-        <v>16</v>
-      </c>
-      <c r="R23">
-        <v>17</v>
-      </c>
-      <c r="S23">
-        <v>18</v>
-      </c>
-      <c r="T23">
-        <v>19</v>
+        <v>117</v>
+      </c>
+      <c r="U21" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{78F473DD-69A3-426A-B9CD-5774C24736D8}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{78F473DD-69A3-426A-B9CD-5774C24736D8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
add: Cambio de nombre de los dtos de FilterDto para las listas
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/clientes.xlsx
+++ b/api/src/main/resources/importaciones/clientes.xlsx
@@ -8,22 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8611FB71-A9F3-47C6-A0DA-DE0D701204D8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D46F94-76DC-4C28-92BE-684ECA8A72CB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="120" yWindow="120" windowWidth="18915" windowHeight="8475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" refMode="R1C1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="130">
-  <si>
-    <t>cliente</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="153">
   <si>
     <t>tipoIdentificacion</t>
   </si>
@@ -370,9 +367,6 @@
     <t>1790715949001</t>
   </si>
   <si>
-    <t>tipoCliente</t>
-  </si>
-  <si>
     <t>S</t>
   </si>
   <si>
@@ -410,6 +404,81 @@
   </si>
   <si>
     <t>Codigo Tercero</t>
+  </si>
+  <si>
+    <t>Nombre Tercero</t>
+  </si>
+  <si>
+    <t>10000000000001</t>
+  </si>
+  <si>
+    <t>10000000000002</t>
+  </si>
+  <si>
+    <t>10000000000003</t>
+  </si>
+  <si>
+    <t>10000000000004</t>
+  </si>
+  <si>
+    <t>10000000000005</t>
+  </si>
+  <si>
+    <t>10000000000006</t>
+  </si>
+  <si>
+    <t>10000000000007</t>
+  </si>
+  <si>
+    <t>10000000000008</t>
+  </si>
+  <si>
+    <t>10000000000009</t>
+  </si>
+  <si>
+    <t>10000000000010</t>
+  </si>
+  <si>
+    <t>10000000000011</t>
+  </si>
+  <si>
+    <t>10000000000012</t>
+  </si>
+  <si>
+    <t>10000000000013</t>
+  </si>
+  <si>
+    <t>10000000000014</t>
+  </si>
+  <si>
+    <t>10000000000015</t>
+  </si>
+  <si>
+    <t>10000000000016</t>
+  </si>
+  <si>
+    <t>10000000000017</t>
+  </si>
+  <si>
+    <t>10000000000018</t>
+  </si>
+  <si>
+    <t>10000000000019</t>
+  </si>
+  <si>
+    <t>10000000000020</t>
+  </si>
+  <si>
+    <t>tipoPersoneria</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>M</t>
   </si>
 </sst>
 </file>
@@ -448,7 +517,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -498,16 +566,20 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -927,685 +999,1062 @@
     <col min="9" max="9" width="31.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.85546875" customWidth="1"/>
     <col min="11" max="11" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.42578125" customWidth="1"/>
     <col min="13" max="13" width="17.42578125" customWidth="1"/>
-    <col min="14" max="19" width="21.85546875" customWidth="1"/>
+    <col min="14" max="14" width="21.85546875" customWidth="1"/>
+    <col min="15" max="16" width="21.85546875" style="1" customWidth="1"/>
+    <col min="17" max="19" width="21.85546875" customWidth="1"/>
     <col min="20" max="21" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="N1" s="6" t="s">
+      <c r="L1" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="P1" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="Q1" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="R1" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="S1" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="R1" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="S1" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="T1" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="U1" s="6" t="s">
-        <v>120</v>
+      <c r="T1" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="3" t="s">
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="K2" t="s">
-        <v>12</v>
-      </c>
       <c r="L2" t="s">
-        <v>121</v>
-      </c>
-      <c r="N2" s="5">
-        <v>10</v>
-      </c>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
+        <v>116</v>
+      </c>
+      <c r="M2">
+        <v>593</v>
+      </c>
+      <c r="N2" s="7">
+        <v>17</v>
+      </c>
+      <c r="O2" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P2" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q2" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="R2" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="S2" s="10" t="s">
+        <v>150</v>
+      </c>
       <c r="T2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>130</v>
       </c>
       <c r="F3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L3" t="s">
-        <v>118</v>
+        <v>119</v>
+      </c>
+      <c r="M3">
+        <v>593</v>
+      </c>
+      <c r="N3">
+        <v>17</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>151</v>
       </c>
       <c r="T3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>40</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L4" t="s">
-        <v>121</v>
+        <v>119</v>
+      </c>
+      <c r="M4">
+        <v>593</v>
+      </c>
+      <c r="N4" s="7">
+        <v>17</v>
+      </c>
+      <c r="O4" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P4" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="U4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>132</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L5" t="s">
-        <v>118</v>
+        <v>119</v>
+      </c>
+      <c r="M5">
+        <v>593</v>
+      </c>
+      <c r="N5" s="7">
+        <v>17</v>
+      </c>
+      <c r="O5" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P5" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>42</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>133</v>
       </c>
       <c r="F6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I6" t="s">
-        <v>103</v>
+        <v>102</v>
+      </c>
+      <c r="L6" t="s">
+        <v>116</v>
+      </c>
+      <c r="M6">
+        <v>593</v>
+      </c>
+      <c r="N6" s="7">
+        <v>17</v>
+      </c>
+      <c r="O6" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P6" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q6" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="R6" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="S6" s="10" t="s">
+        <v>150</v>
       </c>
       <c r="T6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>43</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="F7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I7" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="L7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M7">
+        <v>593</v>
+      </c>
+      <c r="N7" s="7">
+        <v>17</v>
+      </c>
+      <c r="O7" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P7" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="U7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>44</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>135</v>
       </c>
       <c r="F8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I8" t="s">
-        <v>105</v>
+        <v>104</v>
+      </c>
+      <c r="L8" t="s">
+        <v>119</v>
+      </c>
+      <c r="M8">
+        <v>593</v>
+      </c>
+      <c r="N8" s="7">
+        <v>17</v>
+      </c>
+      <c r="O8" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P8" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>45</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="F9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I9" t="s">
-        <v>106</v>
+        <v>105</v>
+      </c>
+      <c r="L9" t="s">
+        <v>119</v>
+      </c>
+      <c r="M9">
+        <v>593</v>
+      </c>
+      <c r="N9" s="7">
+        <v>17</v>
+      </c>
+      <c r="O9" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P9" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T9" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="U9" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>46</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>137</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I10" t="s">
-        <v>107</v>
+        <v>106</v>
+      </c>
+      <c r="L10" t="s">
+        <v>116</v>
+      </c>
+      <c r="M10">
+        <v>593</v>
+      </c>
+      <c r="N10" s="7">
+        <v>17</v>
+      </c>
+      <c r="O10" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P10" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q10" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="R10" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="S10" s="10" t="s">
+        <v>150</v>
       </c>
       <c r="T10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>29</v>
+      <c r="A11" s="6" t="s">
+        <v>28</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>47</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>138</v>
       </c>
       <c r="F11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I11" t="s">
-        <v>108</v>
+        <v>107</v>
+      </c>
+      <c r="L11" t="s">
+        <v>119</v>
+      </c>
+      <c r="M11">
+        <v>593</v>
+      </c>
+      <c r="N11" s="7">
+        <v>17</v>
+      </c>
+      <c r="O11" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P11" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="U11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" s="4"/>
+        <v>17</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>139</v>
+      </c>
       <c r="F12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I12" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="L12" t="s">
+        <v>119</v>
+      </c>
+      <c r="M12">
+        <v>593</v>
+      </c>
+      <c r="N12" s="7">
+        <v>17</v>
+      </c>
+      <c r="O12" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P12" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="F13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I13" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="L13" t="s">
+        <v>119</v>
+      </c>
+      <c r="M13">
+        <v>593</v>
+      </c>
+      <c r="N13" s="7">
+        <v>17</v>
+      </c>
+      <c r="O13" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P13" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>32</v>
+      <c r="A14" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="F14" t="s">
+        <v>68</v>
+      </c>
+      <c r="G14" t="s">
         <v>19</v>
       </c>
-      <c r="C14" t="s">
-        <v>51</v>
-      </c>
-      <c r="F14" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14" t="s">
-        <v>20</v>
-      </c>
       <c r="H14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I14" t="s">
-        <v>109</v>
+        <v>108</v>
+      </c>
+      <c r="L14" t="s">
+        <v>116</v>
+      </c>
+      <c r="M14">
+        <v>593</v>
+      </c>
+      <c r="N14" s="7">
+        <v>17</v>
+      </c>
+      <c r="O14" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P14" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q14" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="R14" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="S14" s="10" t="s">
+        <v>150</v>
       </c>
       <c r="T14" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U14" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>33</v>
+      <c r="A15" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>51</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I15" t="s">
-        <v>110</v>
+        <v>109</v>
+      </c>
+      <c r="L15" t="s">
+        <v>119</v>
+      </c>
+      <c r="M15">
+        <v>593</v>
+      </c>
+      <c r="N15" s="7">
+        <v>17</v>
+      </c>
+      <c r="O15" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P15" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T15" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="U15" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>52</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="F16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I16" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="L16" t="s">
+        <v>119</v>
+      </c>
+      <c r="M16">
+        <v>593</v>
+      </c>
+      <c r="N16" s="7">
+        <v>17</v>
+      </c>
+      <c r="O16" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P16" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T16" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U16" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>53</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I17" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="L17" t="s">
+        <v>119</v>
+      </c>
+      <c r="M17">
+        <v>593</v>
+      </c>
+      <c r="N17" s="7">
+        <v>17</v>
+      </c>
+      <c r="O17" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P17" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T17" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U17" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>54</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>145</v>
       </c>
       <c r="F18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I18" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="L18" t="s">
+        <v>119</v>
+      </c>
+      <c r="M18">
+        <v>593</v>
+      </c>
+      <c r="N18" s="7">
+        <v>17</v>
+      </c>
+      <c r="O18" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P18" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T18" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U18" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C19" t="s">
-        <v>56</v>
+        <v>55</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="F19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I19" t="s">
-        <v>111</v>
+        <v>110</v>
+      </c>
+      <c r="L19" t="s">
+        <v>119</v>
+      </c>
+      <c r="M19">
+        <v>593</v>
+      </c>
+      <c r="N19" s="7">
+        <v>17</v>
+      </c>
+      <c r="O19" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P19" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T19" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U19" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>56</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>147</v>
       </c>
       <c r="F20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I20" t="s">
-        <v>112</v>
+        <v>111</v>
+      </c>
+      <c r="L20" t="s">
+        <v>119</v>
+      </c>
+      <c r="M20">
+        <v>593</v>
+      </c>
+      <c r="N20" s="7">
+        <v>17</v>
+      </c>
+      <c r="O20" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P20" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T20" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U20" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C21" t="s">
-        <v>58</v>
+        <v>57</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="F21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I21" t="s">
-        <v>113</v>
+        <v>112</v>
+      </c>
+      <c r="L21" t="s">
+        <v>119</v>
+      </c>
+      <c r="M21">
+        <v>593</v>
+      </c>
+      <c r="N21" s="7">
+        <v>17</v>
+      </c>
+      <c r="O21" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="P21" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="T21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="U21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>